<commit_message>
Complete AI Study Planner implementation and verification
</commit_message>
<xml_diff>
--- a/testing/reports/AI_Study_Planner_Appium_E2E.xlsx
+++ b/testing/reports/AI_Study_Planner_Appium_E2E.xlsx
@@ -566,7 +566,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Executive Mobile Automation Audit (4-State Pattern) | Executed: 2026-08-19 13:53:17</t>
+          <t>Executive Mobile Automation Audit (4-State Pattern) | Executed: 2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>9.88 seconds</t>
+          <t>9.58 seconds</t>
         </is>
       </c>
       <c r="F10" s="7" t="n"/>
@@ -846,7 +846,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="G23" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="G27" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="G29" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G31" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="G33" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="G35" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="G37" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="G39" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="G41" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="G43" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="G45" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="G47" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="G49" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="G51" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="G53" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="G55" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="G57" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="G59" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="G61" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="G63" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="G64" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="G65" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="G66" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="G67" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="G68" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="G69" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="G71" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="G72" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="G73" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="G74" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="G75" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="G77" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="G78" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="G79" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G80" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="G81" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="G82" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="G83" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="G84" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="G85" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
       </c>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="G87" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="G88" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="G89" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3926,7 +3926,7 @@
       </c>
       <c r="G90" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="G91" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="G92" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="G93" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="G94" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="G95" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="G96" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="G97" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="G98" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="G99" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="G100" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="G101" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="G102" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="G103" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4416,7 @@
       </c>
       <c r="G104" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="G105" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="G106" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="G107" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
       </c>
       <c r="G108" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="G109" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="G110" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="G111" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4696,7 @@
       </c>
       <c r="G112" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4731,7 +4731,7 @@
       </c>
       <c r="G113" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G114" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="G115" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4836,7 +4836,7 @@
       </c>
       <c r="G116" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="G117" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="G118" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="G119" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="G120" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="G121" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="G122" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="G123" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="G124" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="G125" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="G126" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="G127" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="G128" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G129" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="G130" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="G131" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="G132" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="G133" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5466,7 +5466,7 @@
       </c>
       <c r="G134" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="G135" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="G136" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="G137" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5606,7 +5606,7 @@
       </c>
       <c r="G138" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="G139" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5676,7 +5676,7 @@
       </c>
       <c r="G140" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5711,7 +5711,7 @@
       </c>
       <c r="G141" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5746,7 +5746,7 @@
       </c>
       <c r="G142" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5781,7 +5781,7 @@
       </c>
       <c r="G143" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5816,7 +5816,7 @@
       </c>
       <c r="G144" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="G145" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5886,7 +5886,7 @@
       </c>
       <c r="G146" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5921,7 +5921,7 @@
       </c>
       <c r="G147" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5956,7 +5956,7 @@
       </c>
       <c r="G148" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="G149" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6026,7 +6026,7 @@
       </c>
       <c r="G150" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6061,7 +6061,7 @@
       </c>
       <c r="G151" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6096,7 +6096,7 @@
       </c>
       <c r="G152" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6131,7 +6131,7 @@
       </c>
       <c r="G153" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="G154" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="G155" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6236,7 +6236,7 @@
       </c>
       <c r="G156" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="G157" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6306,7 +6306,7 @@
       </c>
       <c r="G158" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6341,7 +6341,7 @@
       </c>
       <c r="G159" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="G160" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="G161" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6446,7 +6446,7 @@
       </c>
       <c r="G162" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6481,7 @@
       </c>
       <c r="G163" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6516,7 +6516,7 @@
       </c>
       <c r="G164" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="G165" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="G166" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6621,7 +6621,7 @@
       </c>
       <c r="G167" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6656,7 +6656,7 @@
       </c>
       <c r="G168" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6691,7 +6691,7 @@
       </c>
       <c r="G169" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="G170" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="G171" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6796,7 +6796,7 @@
       </c>
       <c r="G172" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="G173" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="G174" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="G175" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       </c>
       <c r="G176" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -6971,7 +6971,7 @@
       </c>
       <c r="G177" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="G178" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7041,7 +7041,7 @@
       </c>
       <c r="G179" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7076,7 +7076,7 @@
       </c>
       <c r="G180" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7111,7 +7111,7 @@
       </c>
       <c r="G181" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="G182" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7181,7 @@
       </c>
       <c r="G183" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="G184" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="G185" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7286,7 @@
       </c>
       <c r="G186" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7321,7 +7321,7 @@
       </c>
       <c r="G187" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7356,7 +7356,7 @@
       </c>
       <c r="G188" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7391,7 +7391,7 @@
       </c>
       <c r="G189" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7426,7 +7426,7 @@
       </c>
       <c r="G190" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="G191" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7496,7 +7496,7 @@
       </c>
       <c r="G192" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
       </c>
       <c r="G193" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7566,7 +7566,7 @@
       </c>
       <c r="G194" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7601,7 +7601,7 @@
       </c>
       <c r="G195" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7636,7 +7636,7 @@
       </c>
       <c r="G196" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7671,7 +7671,7 @@
       </c>
       <c r="G197" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="G198" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7741,7 +7741,7 @@
       </c>
       <c r="G199" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7776,7 +7776,7 @@
       </c>
       <c r="G200" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7811,7 +7811,7 @@
       </c>
       <c r="G201" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7846,7 +7846,7 @@
       </c>
       <c r="G202" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7881,7 +7881,7 @@
       </c>
       <c r="G203" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="G204" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7951,7 +7951,7 @@
       </c>
       <c r="G205" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -7986,7 +7986,7 @@
       </c>
       <c r="G206" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8021,7 +8021,7 @@
       </c>
       <c r="G207" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8056,7 +8056,7 @@
       </c>
       <c r="G208" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8091,7 +8091,7 @@
       </c>
       <c r="G209" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="G210" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8161,7 +8161,7 @@
       </c>
       <c r="G211" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8196,7 +8196,7 @@
       </c>
       <c r="G212" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8231,7 +8231,7 @@
       </c>
       <c r="G213" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8266,7 +8266,7 @@
       </c>
       <c r="G214" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="G215" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="G216" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8371,7 +8371,7 @@
       </c>
       <c r="G217" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8406,7 +8406,7 @@
       </c>
       <c r="G218" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="G219" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8476,7 +8476,7 @@
       </c>
       <c r="G220" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8511,7 +8511,7 @@
       </c>
       <c r="G221" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="G222" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="G223" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8616,7 +8616,7 @@
       </c>
       <c r="G224" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8651,7 +8651,7 @@
       </c>
       <c r="G225" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8686,7 +8686,7 @@
       </c>
       <c r="G226" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8721,7 +8721,7 @@
       </c>
       <c r="G227" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8756,7 +8756,7 @@
       </c>
       <c r="G228" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8791,7 +8791,7 @@
       </c>
       <c r="G229" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8826,7 +8826,7 @@
       </c>
       <c r="G230" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8861,7 +8861,7 @@
       </c>
       <c r="G231" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8896,7 +8896,7 @@
       </c>
       <c r="G232" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8931,7 +8931,7 @@
       </c>
       <c r="G233" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -8966,7 +8966,7 @@
       </c>
       <c r="G234" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9001,7 +9001,7 @@
       </c>
       <c r="G235" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9036,7 +9036,7 @@
       </c>
       <c r="G236" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9071,7 +9071,7 @@
       </c>
       <c r="G237" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9106,7 +9106,7 @@
       </c>
       <c r="G238" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9141,7 +9141,7 @@
       </c>
       <c r="G239" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9176,7 @@
       </c>
       <c r="G240" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:16</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9211,7 +9211,7 @@
       </c>
       <c r="G241" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="G242" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9281,7 +9281,7 @@
       </c>
       <c r="G243" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9316,7 @@
       </c>
       <c r="G244" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9351,7 +9351,7 @@
       </c>
       <c r="G245" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9386,7 +9386,7 @@
       </c>
       <c r="G246" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9421,7 +9421,7 @@
       </c>
       <c r="G247" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9456,7 +9456,7 @@
       </c>
       <c r="G248" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9491,7 +9491,7 @@
       </c>
       <c r="G249" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9526,7 +9526,7 @@
       </c>
       <c r="G250" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9561,7 +9561,7 @@
       </c>
       <c r="G251" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9596,7 +9596,7 @@
       </c>
       <c r="G252" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9631,7 +9631,7 @@
       </c>
       <c r="G253" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9666,7 +9666,7 @@
       </c>
       <c r="G254" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9701,7 +9701,7 @@
       </c>
       <c r="G255" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9736,7 +9736,7 @@
       </c>
       <c r="G256" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9771,7 +9771,7 @@
       </c>
       <c r="G257" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="G258" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9841,7 +9841,7 @@
       </c>
       <c r="G259" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="G260" s="11" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>
@@ -9911,7 +9911,7 @@
       </c>
       <c r="G261" s="15" t="inlineStr">
         <is>
-          <t>2026-08-19 13:53:17</t>
+          <t>2026-08-20 15:41:13</t>
         </is>
       </c>
     </row>

</xml_diff>